<commit_message>
bhotange chihaan paati provided
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/nagar bhaipari and estimate misc/bhutange tol khanepani jastaa.xlsx
+++ b/बजेट माग estimate/nagar bhaipari and estimate misc/bhutange tol khanepani jastaa.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B107F568-A3FD-4D43-A1A1-1A11FC206CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBBAC427-7212-4CB5-B11F-2A56CDBF3581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$32</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -178,12 +178,6 @@
   </si>
   <si>
     <t>-MS square pipe of size 1.5"*1.5" and 1.6mm thickness for purlins</t>
-  </si>
-  <si>
-    <t>-MS square pipe of size 2"*2" and 1.6mm thickness for inclined member</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date:2082          </t>
   </si>
   <si>
     <r>
@@ -196,6 +190,9 @@
       </rPr>
       <t xml:space="preserve"> vfg]kfgL 6\ofÍL dfly h:tf 5fpg]</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Date:                  </t>
   </si>
 </sst>
 </file>
@@ -473,21 +470,6 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -509,6 +491,21 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1036,7 +1033,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -1051,113 +1048,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
-      <c r="K3" s="50"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="45"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
-      <c r="J4" s="50"/>
-      <c r="K4" s="50"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+      <c r="H4" s="45"/>
+      <c r="I4" s="45"/>
+      <c r="J4" s="45"/>
+      <c r="K4" s="45"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
-      <c r="H5" s="51"/>
-      <c r="I5" s="51"/>
-      <c r="J5" s="51"/>
-      <c r="K5" s="51"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="46"/>
+      <c r="I5" s="46"/>
+      <c r="J5" s="46"/>
+      <c r="K5" s="46"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="52" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="52"/>
-      <c r="C6" s="52"/>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
+      <c r="A6" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="53" t="s">
+      <c r="H6" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="53"/>
-      <c r="J6" s="53"/>
-      <c r="K6" s="53"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46"/>
-      <c r="F7" s="46"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="47" t="s">
+      <c r="H7" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="I7" s="47"/>
-      <c r="J7" s="47"/>
-      <c r="K7" s="47"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="42"/>
+      <c r="K7" s="42"/>
     </row>
     <row r="8" spans="1:11" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
@@ -1219,39 +1216,37 @@
       <c r="J9" s="38"/>
       <c r="K9" s="13"/>
     </row>
-    <row r="10" spans="1:11" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C10" s="40">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D10" s="29">
-        <f>7/3.281</f>
-        <v>2.1334958854007922</v>
+        <f>(14)/3.281</f>
+        <v>4.2669917708015843</v>
       </c>
       <c r="E10" s="29">
-        <v>2.4300000000000002</v>
+        <v>1.83</v>
       </c>
       <c r="F10" s="29">
         <f t="shared" ref="F10" si="0">PRODUCT(C10:E10)</f>
-        <v>31.10637000914355</v>
+        <v>31.234379762267597</v>
       </c>
       <c r="G10" s="29">
         <f t="shared" ref="G10" si="1">F10</f>
-        <v>31.10637000914355</v>
+        <v>31.234379762267597</v>
       </c>
       <c r="H10" s="38"/>
       <c r="I10" s="38"/>
       <c r="J10" s="38"/>
       <c r="K10" s="28"/>
     </row>
-    <row r="11" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
-      <c r="B11" s="39" t="s">
-        <v>41</v>
-      </c>
+      <c r="B11" s="39"/>
       <c r="C11" s="40">
         <v>4</v>
       </c>
@@ -1276,61 +1271,51 @@
       <c r="K11" s="28"/>
     </row>
     <row r="12" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="39"/>
-      <c r="C12" s="40">
-        <v>4</v>
-      </c>
-      <c r="D12" s="29">
-        <f>(14)/3.281</f>
-        <v>4.2669917708015843</v>
-      </c>
-      <c r="E12" s="29">
-        <v>1.83</v>
-      </c>
-      <c r="F12" s="29">
-        <f t="shared" ref="F12" si="4">PRODUCT(C12:E12)</f>
-        <v>31.234379762267597</v>
-      </c>
-      <c r="G12" s="29">
-        <f t="shared" ref="G12" si="5">F12</f>
-        <v>31.234379762267597</v>
-      </c>
-      <c r="H12" s="38"/>
-      <c r="I12" s="38"/>
-      <c r="J12" s="38"/>
-      <c r="K12" s="28"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="38">
+        <f>SUM(G10:G11)</f>
+        <v>62.468759524535194</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="I12" s="2">
+        <v>182.51</v>
+      </c>
+      <c r="J12" s="38">
+        <f>G12*I12</f>
+        <v>11401.173300822918</v>
+      </c>
+      <c r="K12" s="13"/>
     </row>
     <row r="13" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
       <c r="B13" s="39" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="1"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
-      <c r="G13" s="38">
-        <f>SUM(G11:G12)</f>
-        <v>62.468759524535194</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="I13" s="2">
-        <v>182.51</v>
-      </c>
+      <c r="G13" s="38"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="2"/>
       <c r="J13" s="38">
-        <f>G13*I13</f>
-        <v>11401.173300822918</v>
+        <f>0.13*G12*(1871.42/18.94)</f>
+        <v>802.41220556614235</v>
       </c>
       <c r="K13" s="13"/>
     </row>
     <row r="14" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
-      <c r="B14" s="39" t="s">
-        <v>34</v>
-      </c>
+      <c r="B14" s="39"/>
       <c r="C14" s="12"/>
       <c r="D14" s="1"/>
       <c r="E14" s="13"/>
@@ -1338,15 +1323,16 @@
       <c r="G14" s="38"/>
       <c r="H14" s="14"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="38">
-        <f>0.13*G13*(1871.42/18.94)</f>
-        <v>802.41220556614235</v>
-      </c>
+      <c r="J14" s="38"/>
       <c r="K14" s="13"/>
     </row>
-    <row r="15" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11"/>
-      <c r="B15" s="39"/>
+    <row r="15" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="11">
+        <v>2</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>35</v>
+      </c>
       <c r="C15" s="12"/>
       <c r="D15" s="1"/>
       <c r="E15" s="13"/>
@@ -1357,18 +1343,27 @@
       <c r="J15" s="38"/>
       <c r="K15" s="13"/>
     </row>
-    <row r="16" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="11">
-        <v>2</v>
-      </c>
-      <c r="B16" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="13"/>
+    <row r="16" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="11"/>
+      <c r="B16" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="12">
+        <v>1</v>
+      </c>
+      <c r="D16" s="1">
+        <f>14/3.281</f>
+        <v>4.2669917708015843</v>
+      </c>
+      <c r="E16" s="13">
+        <f>14/3.281</f>
+        <v>4.2669917708015843</v>
+      </c>
       <c r="F16" s="13"/>
-      <c r="G16" s="38"/>
+      <c r="G16" s="19">
+        <f t="shared" ref="G16" si="4">PRODUCT(C16:F16)</f>
+        <v>18.207218772088439</v>
+      </c>
       <c r="H16" s="14"/>
       <c r="I16" s="2"/>
       <c r="J16" s="38"/>
@@ -1377,58 +1372,50 @@
     <row r="17" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
       <c r="B17" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" s="12">
-        <v>1</v>
-      </c>
-      <c r="D17" s="1">
-        <f>14/3.281</f>
-        <v>4.2669917708015843</v>
-      </c>
-      <c r="E17" s="13">
-        <f>14/3.281</f>
-        <v>4.2669917708015843</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="C17" s="12"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="13"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="19">
-        <f t="shared" ref="G17" si="6">PRODUCT(C17:F17)</f>
+      <c r="G17" s="38">
+        <f>SUM(G16:G16)</f>
         <v>18.207218772088439</v>
       </c>
-      <c r="H17" s="14"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="38"/>
+      <c r="H17" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="2">
+        <v>1112.58</v>
+      </c>
+      <c r="J17" s="38">
+        <f>G17*I17</f>
+        <v>20256.987461450153</v>
+      </c>
       <c r="K17" s="13"/>
     </row>
-    <row r="18" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11"/>
-      <c r="B18" s="39" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="38">
-        <f>SUM(G17:G17)</f>
-        <v>18.207218772088439</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="I18" s="2">
-        <v>1112.58</v>
-      </c>
-      <c r="J18" s="38">
-        <f>G18*I18</f>
-        <v>20256.987461450153</v>
-      </c>
-      <c r="K18" s="13"/>
+    <row r="18" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="16"/>
+      <c r="B18" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="15">
+        <f>0.13*G17*7050.67/10</f>
+        <v>1668.8501853374105</v>
+      </c>
+      <c r="K18" s="18"/>
     </row>
     <row r="19" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C19" s="18"/>
       <c r="D19" s="18"/>
@@ -1438,15 +1425,15 @@
       <c r="H19" s="18"/>
       <c r="I19" s="18"/>
       <c r="J19" s="15">
-        <f>0.13*G18*7050.67/10</f>
-        <v>1668.8501853374105</v>
+        <f>0.13*G17*1023.75/10</f>
+        <v>242.31532283303204</v>
       </c>
       <c r="K19" s="18"/>
     </row>
     <row r="20" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="16"/>
       <c r="B20" s="17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="18"/>
@@ -1456,15 +1443,15 @@
       <c r="H20" s="18"/>
       <c r="I20" s="18"/>
       <c r="J20" s="15">
-        <f>0.13*G18*1023.75/10</f>
-        <v>242.31532283303204</v>
+        <f>0.13*G17*348.21/10</f>
+        <v>82.419163432175907</v>
       </c>
       <c r="K20" s="18"/>
     </row>
     <row r="21" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C21" s="18"/>
       <c r="D21" s="18"/>
@@ -1474,16 +1461,14 @@
       <c r="H21" s="18"/>
       <c r="I21" s="18"/>
       <c r="J21" s="15">
-        <f>0.13*G18*348.21/10</f>
-        <v>82.419163432175907</v>
+        <f>0.13*G17*165/10</f>
+        <v>39.054484266129705</v>
       </c>
       <c r="K21" s="18"/>
     </row>
     <row r="22" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
-      <c r="B22" s="17" t="s">
-        <v>40</v>
-      </c>
+      <c r="B22" s="17"/>
       <c r="C22" s="18"/>
       <c r="D22" s="18"/>
       <c r="E22" s="18"/>
@@ -1491,172 +1476,162 @@
       <c r="G22" s="18"/>
       <c r="H22" s="18"/>
       <c r="I22" s="18"/>
-      <c r="J22" s="15">
-        <f>0.13*G18*165/10</f>
-        <v>39.054484266129705</v>
-      </c>
+      <c r="J22" s="15"/>
       <c r="K22" s="18"/>
     </row>
-    <row r="23" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="18"/>
-    </row>
-    <row r="24" spans="1:11" s="9" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11">
-        <v>6</v>
-      </c>
-      <c r="B24" s="20" t="s">
+    <row r="23" spans="1:11" s="9" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="11">
+        <v>3</v>
+      </c>
+      <c r="B23" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C24" s="12">
+      <c r="C23" s="12">
         <v>1</v>
       </c>
+      <c r="D23" s="1"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="14">
+        <f t="shared" ref="G23" si="5">PRODUCT(C23:F23)</f>
+        <v>1</v>
+      </c>
+      <c r="H23" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23" s="2">
+        <v>500</v>
+      </c>
+      <c r="J23" s="14">
+        <f>G23*I23</f>
+        <v>500</v>
+      </c>
+      <c r="K23" s="13"/>
+    </row>
+    <row r="24" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="11"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="12"/>
       <c r="D24" s="1"/>
       <c r="E24" s="13"/>
       <c r="F24" s="13"/>
-      <c r="G24" s="14">
-        <f t="shared" ref="G24" si="7">PRODUCT(C24:F24)</f>
-        <v>1</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="I24" s="2">
-        <v>500</v>
-      </c>
-      <c r="J24" s="14">
-        <f>G24*I24</f>
-        <v>500</v>
-      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="15"/>
       <c r="K24" s="13"/>
     </row>
     <row r="25" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="11"/>
-      <c r="B25" s="21"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="13"/>
-    </row>
-    <row r="26" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="22"/>
-      <c r="B26" s="23" t="s">
+      <c r="A25" s="22"/>
+      <c r="B25" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="24"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15">
-        <f>SUM(J10:J24)</f>
+      <c r="C25" s="24"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15">
+        <f>SUM(J10:J23)</f>
         <v>34993.21212370797</v>
       </c>
-      <c r="K26" s="26"/>
-    </row>
-    <row r="27" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="27"/>
+      <c r="K25" s="26"/>
+    </row>
+    <row r="26" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="27"/>
+      <c r="B27" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="49">
+        <f>J25</f>
+        <v>34993.21212370797</v>
+      </c>
+      <c r="D27" s="50"/>
+      <c r="E27" s="29">
+        <v>100</v>
+      </c>
+      <c r="F27" s="27"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="31"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="33"/>
+    </row>
+    <row r="28" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B28" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="C28" s="41">
-        <f>J26</f>
-        <v>34993.21212370797</v>
-      </c>
-      <c r="D28" s="42"/>
-      <c r="E28" s="29">
-        <v>100</v>
-      </c>
-      <c r="F28" s="27"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="31"/>
-      <c r="J28" s="32"/>
-      <c r="K28" s="33"/>
+        <v>20</v>
+      </c>
+      <c r="C28" s="51">
+        <v>30000</v>
+      </c>
+      <c r="D28" s="52"/>
+      <c r="E28" s="29"/>
     </row>
     <row r="29" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B29" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="C29" s="43">
-        <v>30000</v>
-      </c>
-      <c r="D29" s="44"/>
-      <c r="E29" s="29"/>
+        <v>21</v>
+      </c>
+      <c r="C29" s="51">
+        <f>C28-C31-C32</f>
+        <v>28500</v>
+      </c>
+      <c r="D29" s="52"/>
+      <c r="E29" s="29">
+        <f>C29/C27*100</f>
+        <v>81.444366693880028</v>
+      </c>
     </row>
     <row r="30" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B30" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="43">
-        <f>C29-C32-C33</f>
-        <v>28500</v>
-      </c>
-      <c r="D30" s="44"/>
+        <v>25</v>
+      </c>
+      <c r="C30" s="53">
+        <f>C27-C29</f>
+        <v>6493.21212370797</v>
+      </c>
+      <c r="D30" s="53"/>
       <c r="E30" s="29">
-        <f>C30/C28*100</f>
-        <v>81.444366693880028</v>
+        <f>100-E29</f>
+        <v>18.555633306119972</v>
       </c>
     </row>
     <row r="31" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B31" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="C31" s="45">
-        <f>C28-C30</f>
-        <v>6493.21212370797</v>
-      </c>
-      <c r="D31" s="45"/>
+        <v>22</v>
+      </c>
+      <c r="C31" s="49">
+        <f>C28*0.03</f>
+        <v>900</v>
+      </c>
+      <c r="D31" s="50"/>
       <c r="E31" s="29">
-        <f>100-E30</f>
-        <v>18.555633306119972</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B32" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="C32" s="41">
-        <f>C29*0.03</f>
-        <v>900</v>
-      </c>
-      <c r="D32" s="42"/>
+        <v>23</v>
+      </c>
+      <c r="C32" s="49">
+        <f>C28*0.02</f>
+        <v>600</v>
+      </c>
+      <c r="D32" s="50"/>
       <c r="E32" s="29">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="C33" s="41">
-        <f>C29*0.02</f>
-        <v>600</v>
-      </c>
-      <c r="D33" s="42"/>
-      <c r="E33" s="29">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="H7:K7"/>
     <mergeCell ref="A1:K1"/>
@@ -1666,12 +1641,6 @@
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C32:D32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="80" orientation="portrait" r:id="rId1"/>

</xml_diff>